<commit_message>
Updated code and added files
</commit_message>
<xml_diff>
--- a/Data/A2_DataForAnalysis_PostAutoAndManualExtraction_2026_04/ManualAnnot_ExtractedSents_PosthocRd2.xlsx
+++ b/Data/A2_DataForAnalysis_PostAutoAndManualExtraction_2026_04/ManualAnnot_ExtractedSents_PosthocRd2.xlsx
@@ -5,17 +5,29 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ritwikavps/Desktop/GoogleDriveFiles/research/DARCLEPaper2025/DARCLEPaper2025_ExtractionCode/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ritwikavps/Desktop/GoogleDriveFiles/research/DARCLEPaper2025/DARCLEPaper2025_ExtractionCode/Data/A2_DataForAnalysis_PostAutoAndManualExtraction_2026_04/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA32F3C-BC81-4B43-8FAE-A70CDE9BABE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAA8734-272F-F34A-BBEF-1091D19A2591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -89,7 +101,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -101,12 +113,6 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>

</xml_diff>